<commit_message>
feat(schema): render the Datatype Ontology with its own names and IRIs
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/datatype.xlsx
+++ b/project/excel/datatype.xlsx
@@ -7,14 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Text" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Boolean" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Concept" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Count" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="QuantitativeMeasure" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="QuantitativeRange" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Percent" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="PercentRange" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Boolean" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Concept" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Count" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="QuantitativeMeasure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="QuantitativeRange" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Percent" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PercentRange" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Text" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,6 +441,192 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rdf_value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>vocabulary</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -454,200 +640,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>vocabulary</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>uncertainty</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>uncertainty</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>standard</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>uncertainty</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>uncertainty</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>standard</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>uncertainty</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>